<commit_message>
Fix StoreHub sync PERMISSION_DENIED: eliminate all delete operations
The server-side sync route (/api/storehub/sync) still used the old
delete+recreate pattern that Firestore rules block. Applies the same
deterministic doc ID fix (storehub__branch__dept__date__item) so
re-syncing overwrites existing docs without needing deletes. Also
removes the deleteDoc call on storehub_unmatched — now always setDoc
with items:[] when nothing is unmatched.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/StoreHub SKU Mapping.xlsx
+++ b/StoreHub SKU Mapping.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Current Mapping" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Unmatched SKUs (Review)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Production Config" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,8 +41,32 @@
       <b val="1"/>
       <color rgb="00C00000"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="009CA3AF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -68,8 +93,18 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -77,11 +112,16 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00E5E7EB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -99,6 +139,18 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3153,4 +3205,249 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>⚠️  Fill in each row. 'Portioned Item' must match the exact item name in the stock catalog. Leave 'Yields per Pack' blank if unknown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Raw Material</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Pack Label</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Portioned Item (catalog name)</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Yields per Pack</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Name of the raw supplier item</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>e.g. 500g pack, 1kg bag, block</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Exact name from stock catalog</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Portions produced per 1 pack</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>── Raw Materials ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Wagyu Cubes</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>500g pack</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr"/>
+      <c r="D5" s="11" t="inlineStr"/>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>e.g. Wagyu 150g Portion → 3 per pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>French Fries</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>1kg bag</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr"/>
+      <c r="D6" s="11" t="inlineStr"/>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>e.g. Fries → 8 portions per bag</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Potato Chips</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>1kg bag</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr"/>
+      <c r="D7" s="11" t="inlineStr"/>
+      <c r="E7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Cheese</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>1kg block</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr"/>
+      <c r="D8" s="11" t="inlineStr"/>
+      <c r="E8" s="11" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="12" t="inlineStr"/>
+      <c r="B9" s="12" t="inlineStr"/>
+      <c r="C9" s="12" t="inlineStr"/>
+      <c r="D9" s="12" t="inlineStr"/>
+      <c r="E9" s="12" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="12" t="inlineStr"/>
+      <c r="B10" s="12" t="inlineStr"/>
+      <c r="C10" s="12" t="inlineStr"/>
+      <c r="D10" s="12" t="inlineStr"/>
+      <c r="E10" s="12" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="12" t="inlineStr"/>
+      <c r="B11" s="12" t="inlineStr"/>
+      <c r="C11" s="12" t="inlineStr"/>
+      <c r="D11" s="12" t="inlineStr"/>
+      <c r="E11" s="12" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="12" t="inlineStr"/>
+      <c r="B12" s="12" t="inlineStr"/>
+      <c r="C12" s="12" t="inlineStr"/>
+      <c r="D12" s="12" t="inlineStr"/>
+      <c r="E12" s="12" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="12" t="inlineStr"/>
+      <c r="B13" s="12" t="inlineStr"/>
+      <c r="C13" s="12" t="inlineStr"/>
+      <c r="D13" s="12" t="inlineStr"/>
+      <c r="E13" s="12" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="12" t="inlineStr"/>
+      <c r="B14" s="12" t="inlineStr"/>
+      <c r="C14" s="12" t="inlineStr"/>
+      <c r="D14" s="12" t="inlineStr"/>
+      <c r="E14" s="12" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="12" t="inlineStr"/>
+      <c r="B15" s="12" t="inlineStr"/>
+      <c r="C15" s="12" t="inlineStr"/>
+      <c r="D15" s="12" t="inlineStr"/>
+      <c r="E15" s="12" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="12" t="inlineStr"/>
+      <c r="B16" s="12" t="inlineStr"/>
+      <c r="C16" s="12" t="inlineStr"/>
+      <c r="D16" s="12" t="inlineStr"/>
+      <c r="E16" s="12" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="12" t="inlineStr"/>
+      <c r="B17" s="12" t="inlineStr"/>
+      <c r="C17" s="12" t="inlineStr"/>
+      <c r="D17" s="12" t="inlineStr"/>
+      <c r="E17" s="12" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="12" t="inlineStr"/>
+      <c r="B18" s="12" t="inlineStr"/>
+      <c r="C18" s="12" t="inlineStr"/>
+      <c r="D18" s="12" t="inlineStr"/>
+      <c r="E18" s="12" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="12" t="inlineStr"/>
+      <c r="B19" s="12" t="inlineStr"/>
+      <c r="C19" s="12" t="inlineStr"/>
+      <c r="D19" s="12" t="inlineStr"/>
+      <c r="E19" s="12" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="12" t="inlineStr"/>
+      <c r="B20" s="12" t="inlineStr"/>
+      <c r="C20" s="12" t="inlineStr"/>
+      <c r="D20" s="12" t="inlineStr"/>
+      <c r="E20" s="12" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A4:E4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>